<commit_message>
Fix date-column alignment bug (haga/nagano/shizuoka/minato/iiyama/fukushima amount+reason were shifted); add bundle-purchase continuation-row support; add Aichi/Gifu/Mie region (5 hospitals)
</commit_message>
<xml_diff>
--- a/output/新潟栃木群馬埼玉_赤十字病院_随意契約_X線関連_サマリー.xlsx
+++ b/output/新潟栃木群馬埼玉_赤十字病院_随意契約_X線関連_サマリー.xlsx
@@ -451,11 +451,11 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
-    <col width="30" customWidth="1" min="2" max="2"/>
+    <col width="34" customWidth="1" min="2" max="2"/>
     <col width="14" customWidth="1" min="3" max="3"/>
     <col width="14" customWidth="1" min="4" max="4"/>
     <col width="40" customWidth="1" min="5" max="5"/>
-    <col width="40" customWidth="1" min="6" max="6"/>
+    <col width="44" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -753,7 +753,7 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
-    <col width="26" customWidth="1" min="2" max="2"/>
+    <col width="30" customWidth="1" min="2" max="2"/>
     <col width="36" customWidth="1" min="3" max="3"/>
     <col width="14" customWidth="1" min="4" max="4"/>
     <col width="14" customWidth="1" min="5" max="5"/>
@@ -1053,27 +1053,25 @@
       </c>
       <c r="D7" s="3" t="inlineStr">
         <is>
+          <t>令和7年4月1日</t>
+        </is>
+      </c>
+      <c r="E7" s="5" t="n">
+        <v>6578000</v>
+      </c>
+      <c r="F7" s="3" t="inlineStr">
+        <is>
+          <t>一般撮影（レントゲン）</t>
+        </is>
+      </c>
+      <c r="G7" s="3" t="inlineStr">
+        <is>
+          <t>保守</t>
+        </is>
+      </c>
+      <c r="H7" s="3" t="inlineStr">
+        <is>
           <t>富士フイルムメディカル株式会社北関東支社さいたま市大宮区浅間町2-240</t>
-        </is>
-      </c>
-      <c r="E7" s="3" t="inlineStr">
-        <is>
-          <t>円</t>
-        </is>
-      </c>
-      <c r="F7" s="3" t="inlineStr">
-        <is>
-          <t>一般撮影（レントゲン）</t>
-        </is>
-      </c>
-      <c r="G7" s="3" t="inlineStr">
-        <is>
-          <t>保守</t>
-        </is>
-      </c>
-      <c r="H7" s="3" t="inlineStr">
-        <is>
-          <t>6,578,000</t>
         </is>
       </c>
       <c r="I7" s="3" t="inlineStr">
@@ -1100,27 +1098,25 @@
       </c>
       <c r="D8" s="3" t="inlineStr">
         <is>
+          <t>令和7年4月1日</t>
+        </is>
+      </c>
+      <c r="E8" s="5" t="n">
+        <v>16500000</v>
+      </c>
+      <c r="F8" s="3" t="inlineStr">
+        <is>
+          <t>血管撮影（CVS、アンギオ）</t>
+        </is>
+      </c>
+      <c r="G8" s="3" t="inlineStr">
+        <is>
+          <t>保守</t>
+        </is>
+      </c>
+      <c r="H8" s="3" t="inlineStr">
+        <is>
           <t>日成メディカル宇都宮市問屋町3426-39</t>
-        </is>
-      </c>
-      <c r="E8" s="3" t="inlineStr">
-        <is>
-          <t>円</t>
-        </is>
-      </c>
-      <c r="F8" s="3" t="inlineStr">
-        <is>
-          <t>血管撮影（CVS、アンギオ）</t>
-        </is>
-      </c>
-      <c r="G8" s="3" t="inlineStr">
-        <is>
-          <t>保守</t>
-        </is>
-      </c>
-      <c r="H8" s="3" t="inlineStr">
-        <is>
-          <t>16,500,000</t>
         </is>
       </c>
       <c r="I8" s="3" t="inlineStr">
@@ -1147,27 +1143,25 @@
       </c>
       <c r="D9" s="3" t="inlineStr">
         <is>
+          <t>令和6年5月26日</t>
+        </is>
+      </c>
+      <c r="E9" s="5" t="n">
+        <v>3685000</v>
+      </c>
+      <c r="F9" s="3" t="inlineStr">
+        <is>
+          <t>一般撮影（レントゲン）</t>
+        </is>
+      </c>
+      <c r="G9" s="3" t="inlineStr">
+        <is>
+          <t>製品</t>
+        </is>
+      </c>
+      <c r="H9" s="3" t="inlineStr">
+        <is>
           <t>キヤノンメディカルシステムズ栃木県大田原市下石上1385番地</t>
-        </is>
-      </c>
-      <c r="E9" s="3" t="inlineStr">
-        <is>
-          <t>円</t>
-        </is>
-      </c>
-      <c r="F9" s="3" t="inlineStr">
-        <is>
-          <t>一般撮影（レントゲン）</t>
-        </is>
-      </c>
-      <c r="G9" s="3" t="inlineStr">
-        <is>
-          <t>製品</t>
-        </is>
-      </c>
-      <c r="H9" s="3" t="inlineStr">
-        <is>
-          <t>3,685,000</t>
         </is>
       </c>
       <c r="I9" s="3" t="inlineStr">

</xml_diff>